<commit_message>
Client State Machine WIP
</commit_message>
<xml_diff>
--- a/questions/Assignment6-ClientCommandTableForA7.xlsx
+++ b/questions/Assignment6-ClientCommandTableForA7.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\donav\SimplicityStudio\v5_workspace\ecen5823-assignment6-DonavonFaceyCU\questions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\donav\SimplicityStudio\v5_workspace\ecen5823-assignment7-DonavonFaceyCU\questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241A7BCE-661D-48A7-88F5-339B868C2222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D7DE2BD-4AA8-4FD4-A04C-0F643152CC8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20617" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -275,7 +275,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -286,6 +286,18 @@
       <patternFill patternType="solid">
         <fgColor indexed="9"/>
         <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -420,7 +432,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -469,6 +481,9 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -478,18 +493,20 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" readingOrder="1"/>
-    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1723,23 +1740,23 @@
   <sheetData>
     <row r="1" spans="1:6" ht="14.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="23"/>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="24"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="26"/>
     </row>
     <row r="3" spans="1:6" ht="119.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6"/>
@@ -1787,7 +1804,7 @@
     </row>
     <row r="6" spans="1:6" ht="26.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="8"/>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="27" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="9" t="s">
@@ -1861,7 +1878,7 @@
     </row>
     <row r="12" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4"/>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="28" t="s">
         <v>22</v>
       </c>
       <c r="C12" s="9" t="s">
@@ -1885,7 +1902,7 @@
     </row>
     <row r="14" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4"/>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="28" t="s">
         <v>23</v>
       </c>
       <c r="C14" s="9" t="s">
@@ -1909,7 +1926,7 @@
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4"/>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="29" t="s">
         <v>24</v>
       </c>
       <c r="C16" s="9"/>
@@ -1950,7 +1967,7 @@
       <c r="D19" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="26" t="s">
+      <c r="E19" s="20" t="s">
         <v>28</v>
       </c>
       <c r="F19" s="16"/>
@@ -1974,7 +1991,7 @@
       <c r="D21" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="26" t="s">
+      <c r="E21" s="20" t="s">
         <v>48</v>
       </c>
       <c r="F21" s="12" t="s">
@@ -2038,7 +2055,7 @@
         <v>46</v>
       </c>
       <c r="D27" s="16"/>
-      <c r="E27" s="26" t="s">
+      <c r="E27" s="20" t="s">
         <v>49</v>
       </c>
       <c r="F27" s="16"/>

</xml_diff>